<commit_message>
Revert "Test/e2e UI SquashAndMerge"
This reverts commit b7a51008883ec27657cfbd89d399e2f2a58e1316.
</commit_message>
<xml_diff>
--- a/e-commerce/testData/login.xlsx
+++ b/e-commerce/testData/login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ankit\SeleniumTestNG\e-commerce\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE4F8E60-0B78-4CFE-823E-8C64BD2500E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{716D635B-4D5E-4EFE-AB50-8E281EDB24C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4670" yWindow="1610" windowWidth="14400" windowHeight="8170" xr2:uid="{11688A13-6D12-4117-861E-A32EA8716EC9}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
   <si>
     <t>email</t>
   </si>
@@ -46,6 +46,12 @@
   </si>
   <si>
     <t>Mohan@123</t>
+  </si>
+  <si>
+    <t>Wrong@123</t>
+  </si>
+  <si>
+    <t>wrong@mohan.com</t>
   </si>
 </sst>
 </file>
@@ -81,8 +87,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -397,7 +404,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3482ACDC-737D-4C87-9FF6-72939EA3DF3B}">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:B4"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
@@ -413,10 +420,26 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" t="s">
+      <c r="A2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="1" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+      <c r="A4" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="B4" s="1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Revert "abc revert squash"
This reverts commit 90ef3394384a9f57ec2b2fa842067fea52c1cbcb.
</commit_message>
<xml_diff>
--- a/e-commerce/testData/login.xlsx
+++ b/e-commerce/testData/login.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ankit\SeleniumTestNG\e-commerce\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{716D635B-4D5E-4EFE-AB50-8E281EDB24C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE4F8E60-0B78-4CFE-823E-8C64BD2500E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4670" yWindow="1610" windowWidth="14400" windowHeight="8170" xr2:uid="{11688A13-6D12-4117-861E-A32EA8716EC9}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>email</t>
   </si>
@@ -46,12 +46,6 @@
   </si>
   <si>
     <t>Mohan@123</t>
-  </si>
-  <si>
-    <t>Wrong@123</t>
-  </si>
-  <si>
-    <t>wrong@mohan.com</t>
   </si>
 </sst>
 </file>
@@ -87,9 +81,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3482ACDC-737D-4C87-9FF6-72939EA3DF3B}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
@@ -420,26 +413,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Test/e2e UI Squash and Merge
* Data Update

* e2e Working Automation Script for Positive Scenario

* Jenkinsfile addition

* Ansible added

* Build,Release pipeline integration

* Build and release

* Build and release1

* Build and release2

* Build and release3

* Build and release4

* Pipline Update

* Pipline Update1

* Pipline Update2

* Pipline Update3

* Pipline Update4

* Pipline Update5

* Simplify Jenkins pipeline by removing checkout stage

Removed unnecessary checkout stage and git tool.

* Pipline Update6

* Pipline Update8

* Pipline Update9

* Pipline Update9

* Pipline Update10

* Pipline Update11

* Pipline Update12

* Pipline Update14

* ignore

* Revert "Test/e2e UI SquashAndMerge"

This reverts commit b7a51008883ec27657cfbd89d399e2f2a58e1316.

* commited one duplicate line

* ignore update?

* data update

* successful built

* updated

* Revert "abc revert squash"

This reverts commit 90ef3394384a9f57ec2b2fa842067fea52c1cbcb.

* test

* test done
</commit_message>
<xml_diff>
--- a/e-commerce/testData/login.xlsx
+++ b/e-commerce/testData/login.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Ankit\SeleniumTestNG\e-commerce\testData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{716D635B-4D5E-4EFE-AB50-8E281EDB24C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C0A728F-3675-4052-8726-A80BD3BCE9A7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="4670" yWindow="1610" windowWidth="14400" windowHeight="8170" xr2:uid="{11688A13-6D12-4117-861E-A32EA8716EC9}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>email</t>
   </si>
@@ -46,12 +46,6 @@
   </si>
   <si>
     <t>Mohan@123</t>
-  </si>
-  <si>
-    <t>Wrong@123</t>
-  </si>
-  <si>
-    <t>wrong@mohan.com</t>
   </si>
 </sst>
 </file>
@@ -87,9 +81,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -404,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3482ACDC-737D-4C87-9FF6-72939EA3DF3B}">
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18.7265625" bestFit="1" customWidth="1"/>
@@ -420,26 +413,10 @@
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A2" s="1" t="s">
+      <c r="A2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="1" t="s">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A3" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
-      <c r="A4" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="B4" s="1" t="s">
+      <c r="B2" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>